<commit_message>
fix 2 error file
</commit_message>
<xml_diff>
--- a/Chất thải rắn được xử lý bình quân một ngày phân theo địa phương chia theo Địa phương, Năm và Chất thải rắn.xlsx
+++ b/Chất thải rắn được xử lý bình quân một ngày phân theo địa phương chia theo Địa phương, Năm và Chất thải rắn.xlsx
@@ -16,10 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="75">
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="74">
   <si>
     <t>Tổng lượng chất thải rắn thông thường được thu gom</t>
   </si>
@@ -274,11 +271,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -493,75 +493,85 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="46.71"/>
-    <col customWidth="1" min="2" max="2" width="98.43"/>
-    <col customWidth="1" min="3" max="3" width="46.71"/>
+    <col customWidth="1" min="2" max="2" width="49.29"/>
+    <col customWidth="1" min="3" max="3" width="31.29"/>
     <col customWidth="1" min="4" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
       <c r="B1" s="1">
         <v>2015.0</v>
       </c>
-      <c r="C1" s="1">
+      <c r="D1" s="1">
         <v>2016.0</v>
       </c>
-      <c r="D1" s="1">
+      <c r="F1" s="1">
         <v>2017.0</v>
       </c>
-      <c r="E1" s="1">
+      <c r="H1" s="1">
         <v>2018.0</v>
       </c>
-      <c r="F1" s="1">
+      <c r="J1" s="1">
         <v>2019.0</v>
       </c>
-      <c r="G1" s="1">
+      <c r="L1" s="1">
         <v>2020.0</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1">
         <v>32.415</v>
@@ -602,7 +612,7 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1">
         <v>9.4</v>
@@ -643,7 +653,7 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1">
         <v>5.4</v>
@@ -684,7 +694,7 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1">
         <v>296.0</v>
@@ -725,13 +735,13 @@
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1">
         <v>300.0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" s="1">
         <v>335.0</v>
@@ -766,7 +776,7 @@
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1">
         <v>737.0</v>
@@ -807,7 +817,7 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="1">
         <v>243.0</v>
@@ -848,7 +858,7 @@
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="1">
         <v>1.408</v>
@@ -889,7 +899,7 @@
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="1">
         <v>257.0</v>
@@ -930,7 +940,7 @@
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="1">
         <v>307.0</v>
@@ -971,7 +981,7 @@
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="1">
         <v>105.0</v>
@@ -1004,15 +1014,15 @@
         <v>77.0</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="1">
         <v>219.0</v>
@@ -1053,7 +1063,7 @@
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="1">
         <v>128.0</v>
@@ -1094,7 +1104,7 @@
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1">
         <v>2.277</v>
@@ -1135,7 +1145,7 @@
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17" s="1">
         <v>147.0</v>
@@ -1176,7 +1186,7 @@
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" s="1">
         <v>63.0</v>
@@ -1209,15 +1219,15 @@
         <v>7.0</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="1">
         <v>68.0</v>
@@ -1229,7 +1239,7 @@
         <v>68.0</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" s="1">
         <v>68.0</v>
@@ -1258,7 +1268,7 @@
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" s="1">
         <v>134.0</v>
@@ -1299,13 +1309,13 @@
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="1">
         <v>182.0</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D21" s="1">
         <v>166.0</v>
@@ -1340,7 +1350,7 @@
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="1">
         <v>196.0</v>
@@ -1381,7 +1391,7 @@
     </row>
     <row r="23" ht="14.25" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23" s="1">
         <v>237.0</v>
@@ -1422,7 +1432,7 @@
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" s="1">
         <v>200.0</v>
@@ -1434,7 +1444,7 @@
         <v>251.0</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F24" s="1">
         <v>253.0</v>
@@ -1463,7 +1473,7 @@
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25" s="1">
         <v>231.0</v>
@@ -1504,7 +1514,7 @@
     </row>
     <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" s="1">
         <v>257.0</v>
@@ -1545,7 +1555,7 @@
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" s="1">
         <v>93.0</v>
@@ -1586,13 +1596,13 @@
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28" s="1">
         <v>68.0</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D28" s="1">
         <v>102.0</v>
@@ -1627,7 +1637,7 @@
     </row>
     <row r="29" ht="14.25" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" s="1">
         <v>277.0</v>
@@ -1660,15 +1670,15 @@
         <v>219.0</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="1">
         <v>123.0</v>
@@ -1709,7 +1719,7 @@
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="1">
         <v>5.143</v>
@@ -1750,7 +1760,7 @@
     </row>
     <row r="32" ht="14.25" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B32" s="1">
         <v>762.0</v>
@@ -1791,7 +1801,7 @@
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B33" s="1">
         <v>640.0</v>
@@ -1832,7 +1842,7 @@
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34" s="1">
         <v>149.0</v>
@@ -1873,7 +1883,7 @@
     </row>
     <row r="35" ht="14.25" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35" s="1">
         <v>204.0</v>
@@ -1906,15 +1916,15 @@
         <v>199.0</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36" s="1">
         <v>187.0</v>
@@ -1955,7 +1965,7 @@
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1">
         <v>289.0</v>
@@ -1996,7 +2006,7 @@
     </row>
     <row r="38" ht="14.25" customHeight="1">
       <c r="A38" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B38" s="1">
         <v>730.0</v>
@@ -2029,15 +2039,15 @@
         <v>1.05</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39" s="1">
         <v>455.0</v>
@@ -2070,15 +2080,15 @@
         <v>606.0</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B40" s="1">
         <v>171.0</v>
@@ -2119,7 +2129,7 @@
     </row>
     <row r="41" ht="14.25" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B41" s="1">
         <v>216.0</v>
@@ -2160,7 +2170,7 @@
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B42" s="1">
         <v>209.0</v>
@@ -2201,7 +2211,7 @@
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B43" s="1">
         <v>475.0</v>
@@ -2242,7 +2252,7 @@
     </row>
     <row r="44" ht="14.25" customHeight="1">
       <c r="A44" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44" s="1">
         <v>177.0</v>
@@ -2283,7 +2293,7 @@
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B45" s="1">
         <v>479.0</v>
@@ -2316,15 +2326,15 @@
         <v>184.0</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B46" s="1">
         <v>1.062</v>
@@ -2365,7 +2375,7 @@
     </row>
     <row r="47" ht="14.25" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B47" s="1">
         <v>145.0</v>
@@ -2406,7 +2416,7 @@
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B48" s="1">
         <v>160.0</v>
@@ -2442,12 +2452,12 @@
         <v>698.0</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B49" s="1">
         <v>363.0</v>
@@ -2488,7 +2498,7 @@
     </row>
     <row r="50" ht="14.25" customHeight="1">
       <c r="A50" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B50" s="1">
         <v>91.0</v>
@@ -2529,7 +2539,7 @@
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B51" s="1">
         <v>303.0</v>
@@ -2570,7 +2580,7 @@
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B52" s="1">
         <v>10.878</v>
@@ -2611,7 +2621,7 @@
     </row>
     <row r="53" ht="14.25" customHeight="1">
       <c r="A53" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B53" s="1">
         <v>206.0</v>
@@ -2652,7 +2662,7 @@
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B54" s="1">
         <v>131.0</v>
@@ -2693,7 +2703,7 @@
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B55" s="1">
         <v>1.074</v>
@@ -2734,7 +2744,7 @@
     </row>
     <row r="56" ht="14.25" customHeight="1">
       <c r="A56" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B56" s="1">
         <v>1.365</v>
@@ -2775,7 +2785,7 @@
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B57" s="1">
         <v>602.0</v>
@@ -2816,7 +2826,7 @@
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B58" s="1">
         <v>7.5</v>
@@ -2849,15 +2859,15 @@
         <v>9.0</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
       <c r="A59" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B59" s="1">
         <v>3.655</v>
@@ -2898,7 +2908,7 @@
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B60" s="1">
         <v>192.0</v>
@@ -2939,7 +2949,7 @@
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B61" s="1">
         <v>332.0</v>
@@ -2951,7 +2961,7 @@
         <v>291.0</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F61" s="1">
         <v>304.0</v>
@@ -2980,7 +2990,7 @@
     </row>
     <row r="62" ht="14.25" customHeight="1">
       <c r="A62" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B62" s="1">
         <v>147.0</v>
@@ -3013,15 +3023,15 @@
         <v>140.0</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M62" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B63" s="1">
         <v>297.0</v>
@@ -3062,7 +3072,7 @@
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B64" s="1">
         <v>142.0</v>
@@ -3103,7 +3113,7 @@
     </row>
     <row r="65" ht="14.25" customHeight="1">
       <c r="A65" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B65" s="1">
         <v>368.0</v>
@@ -3144,7 +3154,7 @@
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B66" s="1">
         <v>349.0</v>
@@ -3185,7 +3195,7 @@
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B67" s="1">
         <v>396.0</v>
@@ -3218,15 +3228,15 @@
         <v>548.0</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
       <c r="A68" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B68" s="1">
         <v>650.0</v>
@@ -3267,7 +3277,7 @@
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B69" s="1">
         <v>212.0</v>
@@ -3308,13 +3318,13 @@
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B70" s="1">
         <v>236.0</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D70" s="1">
         <v>288.0</v>
@@ -3349,7 +3359,7 @@
     </row>
     <row r="71" ht="14.25" customHeight="1">
       <c r="A71" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B71" s="1">
         <v>188.0</v>
@@ -3390,7 +3400,7 @@
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B72" s="1">
         <v>147.0</v>

</xml_diff>